<commit_message>
Listas de precios actualizadas desde Gescom (14/10/2026 11:45)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -10776,7 +10776,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 01/10/2026</t>
+          <t xml:space="preserve">Vigencia: 14/10/2026</t>
         </is>
       </c>
     </row>
@@ -11289,86 +11289,81 @@
     </row>
     <row r="28">
       <c r="A28" s="4">
-        <v>5410003</v>
+        <v>5410002</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JUGO DE LIMON 12X1L MENOYO</t>
-        </is>
-      </c>
-      <c r="C28" s="4">
-        <v>12</v>
-      </c>
-      <c r="D28" s="5">
-        <v>35743.74</v>
-      </c>
+          <t xml:space="preserve">VINAGRE DE ALCOHOL 12X1L MENOYO</t>
+        </is>
+      </c>
+      <c r="C28" s="4"/>
+      <c r="D28" s="5"/>
       <c r="E28" s="5">
-        <f>IF(C28&gt;0,D28/C28,"")</f>
-        <v>2978.645</v>
+        <v>15192.87</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4">
-        <v>5412061</v>
+        <v>5410003</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACEITE DE MANTECA AEROSOL 6X120GR MENOYO</t>
-        </is>
-      </c>
-      <c r="C29" s="4"/>
-      <c r="D29" s="5"/>
+          <t xml:space="preserve">JUGO DE LIMON 12X1L MENOYO</t>
+        </is>
+      </c>
+      <c r="C29" s="4">
+        <v>12</v>
+      </c>
+      <c r="D29" s="5">
+        <v>35743.74</v>
+      </c>
       <c r="E29" s="5">
-        <v>4099.37</v>
+        <f>IF(C29&gt;0,D29/C29,"")</f>
+        <v>2978.645</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4">
-        <v>5425041</v>
+        <v>5412061</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYONESA LIGHT EQUIL 12X250cm3 LIVIAN</t>
-        </is>
-      </c>
-      <c r="C30" s="4">
-        <v>12</v>
-      </c>
-      <c r="D30" s="5">
-        <v>12660.86</v>
-      </c>
+          <t xml:space="preserve">ACEITE DE MANTECA AEROSOL 6X120GR MENOYO</t>
+        </is>
+      </c>
+      <c r="C30" s="4"/>
+      <c r="D30" s="5"/>
       <c r="E30" s="5">
-        <f>IF(C30&gt;0,D30/C30,"")</f>
-        <v>1055.0716666666667</v>
+        <v>4099.37</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4">
-        <v>5425042</v>
+        <v>5425041</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYONESA OLIVA 12X250cm3 LIVIAN</t>
+          <t xml:space="preserve">MAYONESA LIGHT EQUIL 12X250cm3 LIVIAN</t>
         </is>
       </c>
       <c r="C31" s="4">
         <v>12</v>
       </c>
       <c r="D31" s="5">
-        <v>21006.66</v>
+        <v>12660.86</v>
       </c>
       <c r="E31" s="5">
         <f>IF(C31&gt;0,D31/C31,"")</f>
-        <v>1750.555</v>
+        <v>1055.0716666666667</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4">
-        <v>5425043</v>
+        <v>5425042</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYONESA AHUMADA 12X250cm3 LIVIAN</t>
+          <t xml:space="preserve">MAYONESA OLIVA 12X250cm3 LIVIAN</t>
         </is>
       </c>
       <c r="C32" s="4">
@@ -11384,11 +11379,11 @@
     </row>
     <row r="33">
       <c r="A33" s="4">
-        <v>5425044</v>
+        <v>5425043</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYONESA SABOR AJO 12X250cm3 LIVIAN</t>
+          <t xml:space="preserve">MAYONESA AHUMADA 12X250cm3 LIVIAN</t>
         </is>
       </c>
       <c r="C33" s="4">
@@ -11404,96 +11399,116 @@
     </row>
     <row r="34">
       <c r="A34" s="4">
-        <v>5425045</v>
+        <v>5425044</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MOSTAZA 12X250GR LIVIAN</t>
+          <t xml:space="preserve">MAYONESA SABOR AJO 12X250cm3 LIVIAN</t>
         </is>
       </c>
       <c r="C34" s="4">
         <v>12</v>
       </c>
       <c r="D34" s="5">
-        <v>10921.8</v>
+        <v>21006.66</v>
       </c>
       <c r="E34" s="5">
         <f>IF(C34&gt;0,D34/C34,"")</f>
-        <v>910.15</v>
+        <v>1750.555</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4">
-        <v>5425062</v>
+        <v>5425045</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SALSA DE SOJA 6X250ML MENOYO</t>
+          <t xml:space="preserve">MOSTAZA 12X250GR LIVIAN</t>
         </is>
       </c>
       <c r="C35" s="4">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D35" s="5">
-        <v>12579.84</v>
+        <v>10921.8</v>
       </c>
       <c r="E35" s="5">
         <f>IF(C35&gt;0,D35/C35,"")</f>
-        <v>2096.64</v>
+        <v>910.15</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4">
-        <v>5450041</v>
+        <v>5425062</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYONESA LIGHT EQUIL 15X500cm3 LIVIAN</t>
+          <t xml:space="preserve">SALSA DE SOJA 6X250ML MENOYO</t>
         </is>
       </c>
       <c r="C36" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D36" s="5">
-        <v>29082.11</v>
+        <v>12579.84</v>
       </c>
       <c r="E36" s="5">
         <f>IF(C36&gt;0,D36/C36,"")</f>
-        <v>1938.8073333333334</v>
+        <v>2096.64</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4">
-        <v>5450061</v>
+        <v>5450041</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SALSA DE SOJA 6X500ML MENOYO</t>
-        </is>
-      </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="5"/>
+          <t xml:space="preserve">MAYONESA LIGHT EQUIL 15X500cm3 LIVIAN</t>
+        </is>
+      </c>
+      <c r="C37" s="4">
+        <v>15</v>
+      </c>
+      <c r="D37" s="5">
+        <v>29082.11</v>
+      </c>
       <c r="E37" s="5">
-        <v>4096.77</v>
+        <f>IF(C37&gt;0,D37/C37,"")</f>
+        <v>1938.8073333333334</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4">
+        <v>5450061</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SALSA DE SOJA 6X500ML MENOYO</t>
+        </is>
+      </c>
+      <c r="C38" s="4"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5">
+        <v>4096.77</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4">
         <v>54510002</v>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">VINAGRE DE MANZANA 12X1L MENOYO</t>
         </is>
       </c>
-      <c r="C38" s="4">
-        <v>12</v>
-      </c>
-      <c r="D38" s="5">
+      <c r="C39" s="4">
+        <v>12</v>
+      </c>
+      <c r="D39" s="5">
         <v>33911.61</v>
       </c>
-      <c r="E38" s="5">
-        <f>IF(C38&gt;0,D38/C38,"")</f>
+      <c r="E39" s="5">
+        <f>IF(C39&gt;0,D39/C39,"")</f>
         <v>2825.9675</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (14/10/2026 14:44)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -11486,10 +11486,15 @@
           <t xml:space="preserve">SALSA DE SOJA 6X500ML MENOYO</t>
         </is>
       </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="5"/>
+      <c r="C38" s="4">
+        <v>6</v>
+      </c>
+      <c r="D38" s="5">
+        <v>24580.62</v>
+      </c>
       <c r="E38" s="5">
-        <v>4096.77</v>
+        <f>IF(C38&gt;0,D38/C38,"")</f>
+        <v>4096.7699999999995</v>
       </c>
     </row>
     <row r="39">

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (14/10/2026 22:43)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -22,8 +22,7 @@
     <sheet name="POLDITOS" sheetId="18" r:id="rId18"/>
     <sheet name="PORTA HNOS" sheetId="19" r:id="rId19"/>
     <sheet name="PRO DE MAN" sheetId="20" r:id="rId20"/>
-    <sheet name="REFINERIA  DE GRASAS SUDAMERICA" sheetId="21" r:id="rId21"/>
-    <sheet name="RIOSMA" sheetId="22" r:id="rId22"/>
+    <sheet name="RIOSMA" sheetId="21" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,7 +66,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="24">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -200,12 +199,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF455A64"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -249,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -324,9 +317,6 @@
     <xf numFmtId="0" fontId="3" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -16500,7 +16490,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">LISTA DE PRECIOS REFINERIA  DE GRASAS SUDAMERICANA - OCTUBRE 2026 (LISTA 1 - PRECIOS CON IVA)</t>
+          <t xml:space="preserve">LISTA DE PRECIOS RIOSMA - OCTUBRE 2026 (LISTA 1 - PRECIOS CON IVA)</t>
         </is>
       </c>
       <c r="B1" s="1"/>
@@ -16537,116 +16527,6 @@
         </is>
       </c>
       <c r="E3" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Precio por unidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4">
-        <v>450033001</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GRASA VACUNA HAL SACHET 10X500GR</t>
-        </is>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5">
-        <v>1539.97</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4">
-        <v>450033015</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GRASA DE CERDO HAL SACHET 10X500GR</t>
-        </is>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5">
-        <v>1692.55</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4">
-        <v>45412033000</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PRIMICIA PARA UNTAR POTES 250GR</t>
-        </is>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5">
-        <v>1554.12</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="13"/>
-  <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LISTA DE PRECIOS RIOSMA - OCTUBRE 2026 (LISTA 1 - PRECIOS CON IVA)</t>
-        </is>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vigencia: 01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codigo</t>
-        </is>
-      </c>
-      <c r="B3" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Descripcion del producto</t>
-        </is>
-      </c>
-      <c r="C3" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cant. por bulto (unidades)</t>
-        </is>
-      </c>
-      <c r="D3" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Precio por bulto</t>
-        </is>
-      </c>
-      <c r="E3" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">Precio por unidad</t>
         </is>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (15/10/2026 05:48)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -10766,7 +10766,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 14/10/2026</t>
+          <t xml:space="preserve">Vigencia: 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -10850,11 +10850,11 @@
         <v>12</v>
       </c>
       <c r="D6" s="5">
-        <v>10850.94</v>
+        <v>10850.65</v>
       </c>
       <c r="E6" s="5">
         <f>IF(C6&gt;0,D6/C6,"")</f>
-        <v>904.245</v>
+        <v>904.2208333333333</v>
       </c>
     </row>
     <row r="7">
@@ -10890,11 +10890,11 @@
         <v>12</v>
       </c>
       <c r="D8" s="5">
-        <v>16237.28</v>
+        <v>16236.99</v>
       </c>
       <c r="E8" s="5">
         <f>IF(C8&gt;0,D8/C8,"")</f>
-        <v>1353.1066666666668</v>
+        <v>1353.0825</v>
       </c>
     </row>
     <row r="9">
@@ -11190,11 +11190,11 @@
         <v>12</v>
       </c>
       <c r="D23" s="5">
-        <v>8681.22</v>
+        <v>8681.07</v>
       </c>
       <c r="E23" s="5">
         <f>IF(C23&gt;0,D23/C23,"")</f>
-        <v>723.435</v>
+        <v>723.4225</v>
       </c>
     </row>
     <row r="24">
@@ -11283,13 +11283,18 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VINAGRE DE ALCOHOL 12X1L MENOYO</t>
-        </is>
-      </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="5"/>
+          <t xml:space="preserve">VINAGRE DE ALCOHOL 12X1L ALCAZAR</t>
+        </is>
+      </c>
+      <c r="C28" s="4">
+        <v>12</v>
+      </c>
+      <c r="D28" s="5">
+        <v>12989.59</v>
+      </c>
       <c r="E28" s="5">
-        <v>15192.87</v>
+        <f>IF(C28&gt;0,D28/C28,"")</f>
+        <v>1082.4658333333334</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (15/10/2026 11:46)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -9561,7 +9561,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 14/10/2026</t>
+          <t xml:space="preserve">Vigencia: 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -10130,6 +10130,126 @@
       <c r="E30" s="5">
         <f>IF(C30&gt;0,D30/C30,"")</f>
         <v>16661.396666666667</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4">
+        <v>874513</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromat. Gatillo Ropa Limpia 250ML</t>
+        </is>
+      </c>
+      <c r="C31" s="4">
+        <v>12</v>
+      </c>
+      <c r="D31" s="5">
+        <v>30501.37</v>
+      </c>
+      <c r="E31" s="5">
+        <f>IF(C31&gt;0,D31/C31,"")</f>
+        <v>2541.7808333333332</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4">
+        <v>874520</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromat. Gatillo Cony Fresh 250ML</t>
+        </is>
+      </c>
+      <c r="C32" s="4">
+        <v>12</v>
+      </c>
+      <c r="D32" s="5">
+        <v>30501.37</v>
+      </c>
+      <c r="E32" s="5">
+        <f>IF(C32&gt;0,D32/C32,"")</f>
+        <v>2541.7808333333332</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4">
+        <v>874612</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Ropa Limpia 500ml</t>
+        </is>
+      </c>
+      <c r="C33" s="4">
+        <v>12</v>
+      </c>
+      <c r="D33" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E33" s="5">
+        <f>IF(C33&gt;0,D33/C33,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4">
+        <v>874629</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Bubble Candy 500ml</t>
+        </is>
+      </c>
+      <c r="C34" s="4">
+        <v>12</v>
+      </c>
+      <c r="D34" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E34" s="5">
+        <f>IF(C34&gt;0,D34/C34,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4">
+        <v>874698</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Green Bamboo 500ml</t>
+        </is>
+      </c>
+      <c r="C35" s="4">
+        <v>12</v>
+      </c>
+      <c r="D35" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E35" s="5">
+        <f>IF(C35&gt;0,D35/C35,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4">
+        <v>874704</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Cony Fresh 500ml</t>
+        </is>
+      </c>
+      <c r="C36" s="4">
+        <v>12</v>
+      </c>
+      <c r="D36" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E36" s="5">
+        <f>IF(C36&gt;0,D36/C36,"")</f>
+        <v>4574.2316666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (16/10/2026 05:47)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -7676,7 +7676,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 01/10/2026</t>
+          <t xml:space="preserve">Vigencia: 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -8801,10 +8801,15 @@
           <t xml:space="preserve">YOG.BEB.ENT.FRUT/KW. S. X 900GR. MULTVT</t>
         </is>
       </c>
-      <c r="C63" s="4"/>
-      <c r="D63" s="5"/>
+      <c r="C63" s="4">
+        <v>12</v>
+      </c>
+      <c r="D63" s="5">
+        <v>25042.93</v>
+      </c>
       <c r="E63" s="5">
-        <v>2086.91</v>
+        <f>IF(C63&gt;0,D63/C63,"")</f>
+        <v>2086.9108333333334</v>
       </c>
     </row>
     <row r="64">
@@ -9210,11 +9215,11 @@
         <v>12</v>
       </c>
       <c r="D87" s="5">
-        <v>28134.39</v>
+        <v>26379.06</v>
       </c>
       <c r="E87" s="5">
         <f>IF(C87&gt;0,D87/C87,"")</f>
-        <v>2344.5325</v>
+        <v>2198.255</v>
       </c>
     </row>
     <row r="88">
@@ -9561,7 +9566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 15/10/2026</t>
+          <t xml:space="preserve">Vigencia: 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -10138,7 +10143,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aromat. Gatillo Ropa Limpia 250ML</t>
+          <t xml:space="preserve">Aromatiz. Gat. Ropa Limpia 250ml</t>
         </is>
       </c>
       <c r="C31" s="4">
@@ -10158,7 +10163,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aromat. Gatillo Cony Fresh 250ML</t>
+          <t xml:space="preserve">Aromatiz. Gat. Cony Fresh 250ml</t>
         </is>
       </c>
       <c r="C32" s="4">
@@ -10174,81 +10179,361 @@
     </row>
     <row r="33">
       <c r="A33" s="4">
-        <v>874612</v>
+        <v>874537</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aromatiz. Gat. Ropa Limpia 500ml</t>
+          <t xml:space="preserve">Aromatiz. Gat. Bubble Candy 250ml</t>
         </is>
       </c>
       <c r="C33" s="4">
         <v>12</v>
       </c>
       <c r="D33" s="5">
-        <v>54890.78</v>
+        <v>30501.37</v>
       </c>
       <c r="E33" s="5">
         <f>IF(C33&gt;0,D33/C33,"")</f>
-        <v>4574.2316666666666</v>
+        <v>2541.7808333333332</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4">
-        <v>874629</v>
+        <v>874544</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aromatiz. Gat. Bubble Candy 500ml</t>
+          <t xml:space="preserve">Aromatiz. Gat. Green Bamboo 250ml</t>
         </is>
       </c>
       <c r="C34" s="4">
         <v>12</v>
       </c>
       <c r="D34" s="5">
-        <v>54890.78</v>
+        <v>30501.37</v>
       </c>
       <c r="E34" s="5">
         <f>IF(C34&gt;0,D34/C34,"")</f>
-        <v>4574.2316666666666</v>
+        <v>2541.7808333333332</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4">
-        <v>874698</v>
+        <v>874551</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aromatiz. Gat. Green Bamboo 500ml</t>
+          <t xml:space="preserve">Aromatiz. Gat. Coconut Grove 250ml</t>
         </is>
       </c>
       <c r="C35" s="4">
         <v>12</v>
       </c>
       <c r="D35" s="5">
-        <v>54890.78</v>
+        <v>30501.37</v>
       </c>
       <c r="E35" s="5">
         <f>IF(C35&gt;0,D35/C35,"")</f>
-        <v>4574.2316666666666</v>
+        <v>2541.7808333333332</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4">
-        <v>874704</v>
+        <v>874568</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aromatiz. Gat. Cony Fresh 500ml</t>
+          <t xml:space="preserve">Aromatiz. Gat. Exotic Flower 250ml</t>
         </is>
       </c>
       <c r="C36" s="4">
         <v>12</v>
       </c>
       <c r="D36" s="5">
-        <v>54890.78</v>
+        <v>30501.37</v>
       </c>
       <c r="E36" s="5">
         <f>IF(C36&gt;0,D36/C36,"")</f>
+        <v>2541.7808333333332</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4">
+        <v>874575</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Mary Blossom 250ml</t>
+        </is>
+      </c>
+      <c r="C37" s="4">
+        <v>12</v>
+      </c>
+      <c r="D37" s="5">
+        <v>30501.37</v>
+      </c>
+      <c r="E37" s="5">
+        <f>IF(C37&gt;0,D37/C37,"")</f>
+        <v>2541.7808333333332</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4">
+        <v>874582</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Victus 250ml</t>
+        </is>
+      </c>
+      <c r="C38" s="4">
+        <v>12</v>
+      </c>
+      <c r="D38" s="5">
+        <v>30501.37</v>
+      </c>
+      <c r="E38" s="5">
+        <f>IF(C38&gt;0,D38/C38,"")</f>
+        <v>2541.7808333333332</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4">
+        <v>874599</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Santal 250ml</t>
+        </is>
+      </c>
+      <c r="C39" s="4">
+        <v>12</v>
+      </c>
+      <c r="D39" s="5">
+        <v>30501.37</v>
+      </c>
+      <c r="E39" s="5">
+        <f>IF(C39&gt;0,D39/C39,"")</f>
+        <v>2541.7808333333332</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4">
+        <v>874605</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. One Alma 250ml</t>
+        </is>
+      </c>
+      <c r="C40" s="4">
+        <v>12</v>
+      </c>
+      <c r="D40" s="5">
+        <v>30501.37</v>
+      </c>
+      <c r="E40" s="5">
+        <f>IF(C40&gt;0,D40/C40,"")</f>
+        <v>2541.7808333333332</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4">
+        <v>874612</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Ropa Limpia 500ml</t>
+        </is>
+      </c>
+      <c r="C41" s="4">
+        <v>12</v>
+      </c>
+      <c r="D41" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E41" s="5">
+        <f>IF(C41&gt;0,D41/C41,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4">
+        <v>874629</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Bubble Candy 500ml</t>
+        </is>
+      </c>
+      <c r="C42" s="4">
+        <v>12</v>
+      </c>
+      <c r="D42" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E42" s="5">
+        <f>IF(C42&gt;0,D42/C42,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4">
+        <v>874636</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Coconut Grove 500ml</t>
+        </is>
+      </c>
+      <c r="C43" s="4">
+        <v>12</v>
+      </c>
+      <c r="D43" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E43" s="5">
+        <f>IF(C43&gt;0,D43/C43,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4">
+        <v>874643</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Exotic Flower 500ml</t>
+        </is>
+      </c>
+      <c r="C44" s="4">
+        <v>12</v>
+      </c>
+      <c r="D44" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E44" s="5">
+        <f>IF(C44&gt;0,D44/C44,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4">
+        <v>874650</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Mary Blossom 500ml</t>
+        </is>
+      </c>
+      <c r="C45" s="4">
+        <v>12</v>
+      </c>
+      <c r="D45" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E45" s="5">
+        <f>IF(C45&gt;0,D45/C45,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4">
+        <v>874667</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Victus 500ml</t>
+        </is>
+      </c>
+      <c r="C46" s="4">
+        <v>12</v>
+      </c>
+      <c r="D46" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E46" s="5">
+        <f>IF(C46&gt;0,D46/C46,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4">
+        <v>874674</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Santal 500ml</t>
+        </is>
+      </c>
+      <c r="C47" s="4">
+        <v>12</v>
+      </c>
+      <c r="D47" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E47" s="5">
+        <f>IF(C47&gt;0,D47/C47,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4">
+        <v>874681</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. One Alma 500ml</t>
+        </is>
+      </c>
+      <c r="C48" s="4">
+        <v>12</v>
+      </c>
+      <c r="D48" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E48" s="5">
+        <f>IF(C48&gt;0,D48/C48,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4">
+        <v>874698</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Green Bamboo 500ml</t>
+        </is>
+      </c>
+      <c r="C49" s="4">
+        <v>12</v>
+      </c>
+      <c r="D49" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E49" s="5">
+        <f>IF(C49&gt;0,D49/C49,"")</f>
+        <v>4574.2316666666666</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4">
+        <v>874704</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aromatiz. Gat. Cony Fresh 500ml</t>
+        </is>
+      </c>
+      <c r="C50" s="4">
+        <v>12</v>
+      </c>
+      <c r="D50" s="5">
+        <v>54890.78</v>
+      </c>
+      <c r="E50" s="5">
+        <f>IF(C50&gt;0,D50/C50,"")</f>
         <v>4574.2316666666666</v>
       </c>
     </row>
@@ -11446,10 +11731,15 @@
           <t xml:space="preserve">ACEITE DE MANTECA AEROSOL 6X120GR MENOYO</t>
         </is>
       </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="5"/>
+      <c r="C30" s="4">
+        <v>6</v>
+      </c>
+      <c r="D30" s="5">
+        <v>24596.23</v>
+      </c>
       <c r="E30" s="5">
-        <v>4099.37</v>
+        <f>IF(C30&gt;0,D30/C30,"")</f>
+        <v>4099.3716666666669</v>
       </c>
     </row>
     <row r="31">
@@ -11485,11 +11775,11 @@
         <v>12</v>
       </c>
       <c r="D32" s="5">
-        <v>21006.66</v>
+        <v>1750.56</v>
       </c>
       <c r="E32" s="5">
         <f>IF(C32&gt;0,D32/C32,"")</f>
-        <v>1750.555</v>
+        <v>145.88</v>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (19/10/2026 10:18)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -18206,7 +18206,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 01/10/2026</t>
+          <t xml:space="preserve">Vigencia: 19/10/2026</t>
         </is>
       </c>
     </row>
@@ -18270,11 +18270,11 @@
         <v>12</v>
       </c>
       <c r="D5" s="5">
-        <v>52228.72</v>
+        <v>53795.58</v>
       </c>
       <c r="E5" s="5">
         <f>IF(C5&gt;0,D5/C5,"")</f>
-        <v>4352.3933333333334</v>
+        <v>4482.965</v>
       </c>
     </row>
     <row r="6">
@@ -18370,11 +18370,11 @@
         <v>6</v>
       </c>
       <c r="D10" s="5">
-        <v>51104.97</v>
+        <v>52127.08</v>
       </c>
       <c r="E10" s="5">
         <f>IF(C10&gt;0,D10/C10,"")</f>
-        <v>8517.495</v>
+        <v>8687.8466666666664</v>
       </c>
     </row>
     <row r="11">
@@ -18390,11 +18390,11 @@
         <v>6</v>
       </c>
       <c r="D11" s="5">
-        <v>33146.32</v>
+        <v>33809.24</v>
       </c>
       <c r="E11" s="5">
         <f>IF(C11&gt;0,D11/C11,"")</f>
-        <v>5524.3866666666663</v>
+        <v>5634.873333333333</v>
       </c>
     </row>
     <row r="12">
@@ -18430,11 +18430,11 @@
         <v>12</v>
       </c>
       <c r="D13" s="5">
-        <v>46427.75</v>
+        <v>47356.3</v>
       </c>
       <c r="E13" s="5">
         <f>IF(C13&gt;0,D13/C13,"")</f>
-        <v>3868.9791666666665</v>
+        <v>3946.3583333333336</v>
       </c>
     </row>
     <row r="14">
@@ -18450,11 +18450,11 @@
         <v>12</v>
       </c>
       <c r="D14" s="5">
-        <v>91430.83</v>
+        <v>93259.44</v>
       </c>
       <c r="E14" s="5">
         <f>IF(C14&gt;0,D14/C14,"")</f>
-        <v>7619.2358333333332</v>
+        <v>7771.62</v>
       </c>
     </row>
     <row r="15">
@@ -18470,11 +18470,11 @@
         <v>12</v>
       </c>
       <c r="D15" s="5">
-        <v>127610.75</v>
+        <v>130162.97</v>
       </c>
       <c r="E15" s="5">
         <f>IF(C15&gt;0,D15/C15,"")</f>
-        <v>10634.229166666666</v>
+        <v>10846.914166666667</v>
       </c>
     </row>
     <row r="16">
@@ -18490,11 +18490,11 @@
         <v>12</v>
       </c>
       <c r="D16" s="5">
-        <v>87748.96</v>
+        <v>89503.94</v>
       </c>
       <c r="E16" s="5">
         <f>IF(C16&gt;0,D16/C16,"")</f>
-        <v>7312.4133333333339</v>
+        <v>7458.6616666666669</v>
       </c>
     </row>
     <row r="17">
@@ -18570,11 +18570,11 @@
         <v>24</v>
       </c>
       <c r="D20" s="5">
-        <v>46125.2</v>
+        <v>47047.7</v>
       </c>
       <c r="E20" s="5">
         <f>IF(C20&gt;0,D20/C20,"")</f>
-        <v>1921.8833333333332</v>
+        <v>1960.3208333333332</v>
       </c>
     </row>
     <row r="21">
@@ -18590,11 +18590,11 @@
         <v>6</v>
       </c>
       <c r="D21" s="5">
-        <v>41084.91</v>
+        <v>47047.7</v>
       </c>
       <c r="E21" s="5">
         <f>IF(C21&gt;0,D21/C21,"")</f>
-        <v>6847.4850000000006</v>
+        <v>7841.2833333333328</v>
       </c>
     </row>
     <row r="22">
@@ -18610,11 +18610,11 @@
         <v>6</v>
       </c>
       <c r="D22" s="5">
-        <v>76142.37</v>
+        <v>77665.22</v>
       </c>
       <c r="E22" s="5">
         <f>IF(C22&gt;0,D22/C22,"")</f>
-        <v>12690.394999999999</v>
+        <v>12944.203333333333</v>
       </c>
     </row>
     <row r="23">
@@ -18630,11 +18630,11 @@
         <v>24</v>
       </c>
       <c r="D23" s="5">
-        <v>38938.8</v>
+        <v>39717.6</v>
       </c>
       <c r="E23" s="5">
         <f>IF(C23&gt;0,D23/C23,"")</f>
-        <v>1622.45</v>
+        <v>1654.8999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -18650,11 +18650,11 @@
         <v>6</v>
       </c>
       <c r="D24" s="5">
-        <v>57592.37</v>
+        <v>58744.22</v>
       </c>
       <c r="E24" s="5">
         <f>IF(C24&gt;0,D24/C24,"")</f>
-        <v>9598.7283333333344</v>
+        <v>9790.7033333333329</v>
       </c>
     </row>
     <row r="25">
@@ -18670,11 +18670,11 @@
         <v>12</v>
       </c>
       <c r="D25" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E25" s="5">
         <f>IF(C25&gt;0,D25/C25,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="26">
@@ -18690,11 +18690,11 @@
         <v>12</v>
       </c>
       <c r="D26" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E26" s="5">
         <f>IF(C26&gt;0,D26/C26,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="27">
@@ -18710,11 +18710,11 @@
         <v>12</v>
       </c>
       <c r="D27" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E27" s="5">
         <f>IF(C27&gt;0,D27/C27,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="28">
@@ -18730,11 +18730,11 @@
         <v>12</v>
       </c>
       <c r="D28" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E28" s="5">
         <f>IF(C28&gt;0,D28/C28,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="29">
@@ -18750,11 +18750,11 @@
         <v>12</v>
       </c>
       <c r="D29" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E29" s="5">
         <f>IF(C29&gt;0,D29/C29,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="30">
@@ -18770,11 +18770,11 @@
         <v>12</v>
       </c>
       <c r="D30" s="5">
-        <v>41089.19</v>
+        <v>41910.99</v>
       </c>
       <c r="E30" s="5">
         <f>IF(C30&gt;0,D30/C30,"")</f>
-        <v>3424.0991666666669</v>
+        <v>3492.5825</v>
       </c>
     </row>
     <row r="31">
@@ -18790,11 +18790,11 @@
         <v>12</v>
       </c>
       <c r="D31" s="5">
-        <v>41089.19</v>
+        <v>41910.99</v>
       </c>
       <c r="E31" s="5">
         <f>IF(C31&gt;0,D31/C31,"")</f>
-        <v>3424.0991666666669</v>
+        <v>3492.5825</v>
       </c>
     </row>
     <row r="32">
@@ -18810,11 +18810,11 @@
         <v>12</v>
       </c>
       <c r="D32" s="5">
-        <v>41089.19</v>
+        <v>41910.99</v>
       </c>
       <c r="E32" s="5">
         <f>IF(C32&gt;0,D32/C32,"")</f>
-        <v>3424.0991666666669</v>
+        <v>3492.5825</v>
       </c>
     </row>
     <row r="33">
@@ -18830,11 +18830,11 @@
         <v>12</v>
       </c>
       <c r="D33" s="5">
-        <v>41089.19</v>
+        <v>41910.99</v>
       </c>
       <c r="E33" s="5">
         <f>IF(C33&gt;0,D33/C33,"")</f>
-        <v>3424.0991666666669</v>
+        <v>3492.5825</v>
       </c>
     </row>
     <row r="34">
@@ -18850,11 +18850,11 @@
         <v>12</v>
       </c>
       <c r="D34" s="5">
-        <v>41089.19</v>
+        <v>41910.99</v>
       </c>
       <c r="E34" s="5">
         <f>IF(C34&gt;0,D34/C34,"")</f>
-        <v>3424.0991666666669</v>
+        <v>3492.5825</v>
       </c>
     </row>
     <row r="35">
@@ -18870,11 +18870,11 @@
         <v>12</v>
       </c>
       <c r="D35" s="5">
-        <v>41089.19</v>
+        <v>41910.99</v>
       </c>
       <c r="E35" s="5">
         <f>IF(C35&gt;0,D35/C35,"")</f>
-        <v>3424.0991666666669</v>
+        <v>3492.5825</v>
       </c>
     </row>
     <row r="36">
@@ -18890,11 +18890,11 @@
         <v>24</v>
       </c>
       <c r="D36" s="5">
-        <v>45849.9</v>
+        <v>46766.89</v>
       </c>
       <c r="E36" s="5">
         <f>IF(C36&gt;0,D36/C36,"")</f>
-        <v>1910.4125000000001</v>
+        <v>1948.6204166666666</v>
       </c>
     </row>
     <row r="37">
@@ -18910,11 +18910,11 @@
         <v>24</v>
       </c>
       <c r="D37" s="5">
-        <v>45849.9</v>
+        <v>46766.89</v>
       </c>
       <c r="E37" s="5">
         <f>IF(C37&gt;0,D37/C37,"")</f>
-        <v>1910.4125000000001</v>
+        <v>1948.6204166666666</v>
       </c>
     </row>
     <row r="38">
@@ -18930,11 +18930,11 @@
         <v>24</v>
       </c>
       <c r="D38" s="5">
-        <v>45849.9</v>
+        <v>46766.89</v>
       </c>
       <c r="E38" s="5">
         <f>IF(C38&gt;0,D38/C38,"")</f>
-        <v>1910.4125000000001</v>
+        <v>1948.6204166666666</v>
       </c>
     </row>
     <row r="39">
@@ -18950,11 +18950,11 @@
         <v>24</v>
       </c>
       <c r="D39" s="5">
-        <v>45849.9</v>
+        <v>46766.89</v>
       </c>
       <c r="E39" s="5">
         <f>IF(C39&gt;0,D39/C39,"")</f>
-        <v>1910.4125000000001</v>
+        <v>1948.6204166666666</v>
       </c>
     </row>
     <row r="40">
@@ -18970,11 +18970,11 @@
         <v>24</v>
       </c>
       <c r="D40" s="5">
-        <v>45849.9</v>
+        <v>46766.89</v>
       </c>
       <c r="E40" s="5">
         <f>IF(C40&gt;0,D40/C40,"")</f>
-        <v>1910.4125000000001</v>
+        <v>1948.6204166666666</v>
       </c>
     </row>
     <row r="41">
@@ -18990,11 +18990,11 @@
         <v>6</v>
       </c>
       <c r="D41" s="5">
-        <v>54460.01</v>
+        <v>55549.19</v>
       </c>
       <c r="E41" s="5">
         <f>IF(C41&gt;0,D41/C41,"")</f>
-        <v>9076.6683333333331</v>
+        <v>9258.1983333333337</v>
       </c>
     </row>
     <row r="42">
@@ -19010,11 +19010,11 @@
         <v>24</v>
       </c>
       <c r="D42" s="5">
-        <v>53484.23</v>
+        <v>54553.91</v>
       </c>
       <c r="E42" s="5">
         <f>IF(C42&gt;0,D42/C42,"")</f>
-        <v>2228.5095833333335</v>
+        <v>2273.0795833333336</v>
       </c>
     </row>
     <row r="43">
@@ -19030,11 +19030,11 @@
         <v>12</v>
       </c>
       <c r="D43" s="5">
-        <v>116887.69</v>
+        <v>119225.45</v>
       </c>
       <c r="E43" s="5">
         <f>IF(C43&gt;0,D43/C43,"")</f>
-        <v>9740.6408333333329</v>
+        <v>9935.4541666666664</v>
       </c>
     </row>
     <row r="44">
@@ -19050,11 +19050,11 @@
         <v>12</v>
       </c>
       <c r="D44" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E44" s="5">
         <f>IF(C44&gt;0,D44/C44,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="45">
@@ -19070,11 +19070,11 @@
         <v>12</v>
       </c>
       <c r="D45" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E45" s="5">
         <f>IF(C45&gt;0,D45/C45,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="46">
@@ -19090,11 +19090,11 @@
         <v>24</v>
       </c>
       <c r="D46" s="5">
-        <v>45849.9</v>
+        <v>46766.89</v>
       </c>
       <c r="E46" s="5">
         <f>IF(C46&gt;0,D46/C46,"")</f>
-        <v>1910.4125000000001</v>
+        <v>1948.6204166666666</v>
       </c>
     </row>
     <row r="47">
@@ -19110,11 +19110,11 @@
         <v>12</v>
       </c>
       <c r="D47" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E47" s="5">
         <f>IF(C47&gt;0,D47/C47,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="48">
@@ -19130,11 +19130,11 @@
         <v>12</v>
       </c>
       <c r="D48" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E48" s="5">
         <f>IF(C48&gt;0,D48/C48,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="49">
@@ -19150,11 +19150,11 @@
         <v>12</v>
       </c>
       <c r="D49" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E49" s="5">
         <f>IF(C49&gt;0,D49/C49,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="50">
@@ -19170,11 +19170,11 @@
         <v>12</v>
       </c>
       <c r="D50" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E50" s="5">
         <f>IF(C50&gt;0,D50/C50,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="51">
@@ -19190,11 +19190,11 @@
         <v>12</v>
       </c>
       <c r="D51" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E51" s="5">
         <f>IF(C51&gt;0,D51/C51,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="52">
@@ -19210,11 +19210,11 @@
         <v>12</v>
       </c>
       <c r="D52" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E52" s="5">
         <f>IF(C52&gt;0,D52/C52,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="53">
@@ -19230,11 +19230,11 @@
         <v>12</v>
       </c>
       <c r="D53" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E53" s="5">
         <f>IF(C53&gt;0,D53/C53,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="54">
@@ -19250,11 +19250,11 @@
         <v>12</v>
       </c>
       <c r="D54" s="5">
-        <v>23765.08</v>
+        <v>24240.38</v>
       </c>
       <c r="E54" s="5">
         <f>IF(C54&gt;0,D54/C54,"")</f>
-        <v>1980.4233333333334</v>
+        <v>2020.0316666666668</v>
       </c>
     </row>
     <row r="55">
@@ -19290,11 +19290,11 @@
         <v>12</v>
       </c>
       <c r="D56" s="5">
-        <v>35450.64</v>
+        <v>36159.65</v>
       </c>
       <c r="E56" s="5">
         <f>IF(C56&gt;0,D56/C56,"")</f>
-        <v>2954.22</v>
+        <v>3013.3041666666668</v>
       </c>
     </row>
     <row r="57">
@@ -19310,11 +19310,11 @@
         <v>12</v>
       </c>
       <c r="D57" s="5">
-        <v>14185.1</v>
+        <v>14468.8</v>
       </c>
       <c r="E57" s="5">
         <f>IF(C57&gt;0,D57/C57,"")</f>
-        <v>1182.0916666666667</v>
+        <v>1205.7333333333333</v>
       </c>
     </row>
     <row r="58">
@@ -19330,11 +19330,11 @@
         <v>12</v>
       </c>
       <c r="D58" s="5">
-        <v>14185.1</v>
+        <v>14468.8</v>
       </c>
       <c r="E58" s="5">
         <f>IF(C58&gt;0,D58/C58,"")</f>
-        <v>1182.0916666666667</v>
+        <v>1205.7333333333333</v>
       </c>
     </row>
     <row r="59">
@@ -19350,11 +19350,11 @@
         <v>12</v>
       </c>
       <c r="D59" s="5">
-        <v>14185.1</v>
+        <v>14468.8</v>
       </c>
       <c r="E59" s="5">
         <f>IF(C59&gt;0,D59/C59,"")</f>
-        <v>1182.0916666666667</v>
+        <v>1205.7333333333333</v>
       </c>
     </row>
     <row r="60">
@@ -19370,11 +19370,11 @@
         <v>12</v>
       </c>
       <c r="D60" s="5">
-        <v>14185.1</v>
+        <v>14468.8</v>
       </c>
       <c r="E60" s="5">
         <f>IF(C60&gt;0,D60/C60,"")</f>
-        <v>1182.0916666666667</v>
+        <v>1205.7333333333333</v>
       </c>
     </row>
     <row r="61">
@@ -19390,11 +19390,11 @@
         <v>12</v>
       </c>
       <c r="D61" s="5">
-        <v>14185.1</v>
+        <v>14468.8</v>
       </c>
       <c r="E61" s="5">
         <f>IF(C61&gt;0,D61/C61,"")</f>
-        <v>1182.0916666666667</v>
+        <v>1205.7333333333333</v>
       </c>
     </row>
     <row r="62">
@@ -19430,11 +19430,11 @@
         <v>24</v>
       </c>
       <c r="D63" s="5">
-        <v>42118.81</v>
+        <v>42961.18</v>
       </c>
       <c r="E63" s="5">
         <f>IF(C63&gt;0,D63/C63,"")</f>
-        <v>1754.9504166666666</v>
+        <v>1790.0491666666667</v>
       </c>
     </row>
     <row r="64">
@@ -19470,11 +19470,11 @@
         <v>12</v>
       </c>
       <c r="D65" s="5">
-        <v>41089.19</v>
+        <v>41910.99</v>
       </c>
       <c r="E65" s="5">
         <f>IF(C65&gt;0,D65/C65,"")</f>
-        <v>3424.0991666666669</v>
+        <v>3492.5825</v>
       </c>
     </row>
     <row r="66">
@@ -19570,11 +19570,11 @@
         <v>12</v>
       </c>
       <c r="D70" s="5">
-        <v>91430.83</v>
+        <v>93259.44</v>
       </c>
       <c r="E70" s="5">
         <f>IF(C70&gt;0,D70/C70,"")</f>
-        <v>7619.2358333333332</v>
+        <v>7771.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (19/10/2026 11:37)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -7676,7 +7676,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 16/10/2026</t>
+          <t xml:space="preserve">Vigencia: 19/10/2026</t>
         </is>
       </c>
     </row>
@@ -9155,11 +9155,11 @@
         <v>12</v>
       </c>
       <c r="D84" s="5">
-        <v>22179.3</v>
+        <v>20386.08</v>
       </c>
       <c r="E84" s="5">
         <f>IF(C84&gt;0,D84/C84,"")</f>
-        <v>1848.2749999999999</v>
+        <v>1698.8400000000001</v>
       </c>
     </row>
     <row r="85">
@@ -9175,11 +9175,11 @@
         <v>12</v>
       </c>
       <c r="D85" s="5">
-        <v>22179.3</v>
+        <v>20386.08</v>
       </c>
       <c r="E85" s="5">
         <f>IF(C85&gt;0,D85/C85,"")</f>
-        <v>1848.2749999999999</v>
+        <v>1698.8400000000001</v>
       </c>
     </row>
     <row r="86">
@@ -9195,11 +9195,11 @@
         <v>12</v>
       </c>
       <c r="D86" s="5">
-        <v>27804.63</v>
+        <v>22019.13</v>
       </c>
       <c r="E86" s="5">
         <f>IF(C86&gt;0,D86/C86,"")</f>
-        <v>2317.0525000000002</v>
+        <v>1834.9275</v>
       </c>
     </row>
     <row r="87">
@@ -9215,11 +9215,11 @@
         <v>12</v>
       </c>
       <c r="D87" s="5">
-        <v>26379.06</v>
+        <v>24232.43</v>
       </c>
       <c r="E87" s="5">
         <f>IF(C87&gt;0,D87/C87,"")</f>
-        <v>2198.255</v>
+        <v>2019.3691666666666</v>
       </c>
     </row>
     <row r="88">
@@ -9566,7 +9566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 16/10/2026</t>
+          <t xml:space="preserve">Vigencia: 19/10/2026</t>
         </is>
       </c>
     </row>
@@ -18587,14 +18587,14 @@
         </is>
       </c>
       <c r="C21" s="4">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D21" s="5">
         <v>47047.7</v>
       </c>
       <c r="E21" s="5">
         <f>IF(C21&gt;0,D21/C21,"")</f>
-        <v>7841.2833333333328</v>
+        <v>1960.3208333333332</v>
       </c>
     </row>
     <row r="22">
@@ -19499,81 +19499,21 @@
     </row>
     <row r="67">
       <c r="A67" s="4">
-        <v>39014866</v>
+        <v>39014996</v>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1882 FERNET CON POMELO 7 473mlx6x4</t>
+          <t xml:space="preserve">Martini Rosso 16° 12x995ml</t>
         </is>
       </c>
       <c r="C67" s="4">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D67" s="5">
-        <v>37989.09</v>
+        <v>93259.44</v>
       </c>
       <c r="E67" s="5">
         <f>IF(C67&gt;0,D67/C67,"")</f>
-        <v>1582.8787499999999</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4">
-        <v>39014882</v>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gancia LIMA LIMON ONE 4x6x473</t>
-        </is>
-      </c>
-      <c r="C68" s="4">
-        <v>24</v>
-      </c>
-      <c r="D68" s="5">
-        <v>51692.42</v>
-      </c>
-      <c r="E68" s="5">
-        <f>IF(C68&gt;0,D68/C68,"")</f>
-        <v>2153.8508333333334</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="4">
-        <v>39014884</v>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DR LEMON RED BERRIES 5% 4x6x473</t>
-        </is>
-      </c>
-      <c r="C69" s="4">
-        <v>24</v>
-      </c>
-      <c r="D69" s="5">
-        <v>45849.9</v>
-      </c>
-      <c r="E69" s="5">
-        <f>IF(C69&gt;0,D69/C69,"")</f>
-        <v>1910.4125000000001</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4">
-        <v>39014996</v>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Martini Rosso 16° 12x995ml</t>
-        </is>
-      </c>
-      <c r="C70" s="4">
-        <v>12</v>
-      </c>
-      <c r="D70" s="5">
-        <v>93259.44</v>
-      </c>
-      <c r="E70" s="5">
-        <f>IF(C70&gt;0,D70/C70,"")</f>
         <v>7771.62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (20/10/2026 05:47)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -351,7 +351,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 14/10/2026</t>
+          <t xml:space="preserve">Vigencia: 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -2840,11 +2840,11 @@
         <v>54</v>
       </c>
       <c r="E111" s="5">
-        <v>55450.42</v>
+        <v>54222.36</v>
       </c>
       <c r="F111" s="5">
         <f>IF(D111&gt;0,E111/D111,"")</f>
-        <v>1026.8596296296296</v>
+        <v>1004.1177777777777</v>
       </c>
     </row>
     <row r="112">

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (21/10/2026 05:49)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -17371,10 +17371,15 @@
           <t xml:space="preserve">AF BIC SOLEIL CTL X12</t>
         </is>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="5"/>
+      <c r="C14" s="4">
+        <v>24</v>
+      </c>
+      <c r="D14" s="5">
+        <v>391305.58</v>
+      </c>
       <c r="E14" s="5">
-        <v>16304.4</v>
+        <f>IF(C14&gt;0,D14/C14,"")</f>
+        <v>16304.399166666668</v>
       </c>
     </row>
     <row r="15">
@@ -18206,7 +18211,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 19/10/2026</t>
+          <t xml:space="preserve">Vigencia: 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -19499,21 +19504,41 @@
     </row>
     <row r="67">
       <c r="A67" s="4">
-        <v>39014996</v>
+        <v>39014884</v>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Martini Rosso 16° 12x995ml</t>
+          <t xml:space="preserve">DR LEMON RED BERRIES 5% 4x6x473</t>
         </is>
       </c>
       <c r="C67" s="4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D67" s="5">
-        <v>93259.44</v>
+        <v>46766.89</v>
       </c>
       <c r="E67" s="5">
         <f>IF(C67&gt;0,D67/C67,"")</f>
+        <v>1948.6204166666666</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4">
+        <v>39014996</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Martini Rosso 16° 12x995ml</t>
+        </is>
+      </c>
+      <c r="C68" s="4">
+        <v>12</v>
+      </c>
+      <c r="D68" s="5">
+        <v>93259.44</v>
+      </c>
+      <c r="E68" s="5">
+        <f>IF(C68&gt;0,D68/C68,"")</f>
         <v>7771.62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (21/10/2026 11:46)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -3933,7 +3933,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GARAPIÑADAS DE MANÍ</t>
+          <t xml:space="preserve">GARRAPIÑADAS DE MANÍ</t>
         </is>
       </c>
       <c r="C53" s="4"/>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GARAPIÑADA DE MANI NAMUR 36X60GR</t>
+          <t xml:space="preserve">GARRAPIÑADAS DE MANI NAMUR 36X60GR</t>
         </is>
       </c>
       <c r="C54" s="4">
@@ -6668,7 +6668,7 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GARAPIÑADAS DE MANÍ 36X80GR</t>
+          <t xml:space="preserve">GARRAPIÑADAS DE MANÍ 36X80GR</t>
         </is>
       </c>
       <c r="C211" s="4">
@@ -6688,7 +6688,7 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GARAPIÑADAS DE MANÍ 36X100GR</t>
+          <t xml:space="preserve">GARRAPIÑADAS DE MANÍ 36X100GR</t>
         </is>
       </c>
       <c r="C212" s="4">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GARAPIÑADAS DE ALMENDRAS</t>
+          <t xml:space="preserve">GARRAPIÑADAS DE ALMENDRAS</t>
         </is>
       </c>
       <c r="C215" s="4"/>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GARAPIÑADAS DE MANÍ BAÑADA CON CHOCOLATE</t>
+          <t xml:space="preserve">GARRAPIÑADAS DE MANÍ BAÑADA CON CHOCOLATE</t>
         </is>
       </c>
       <c r="C219" s="4"/>
@@ -13326,7 +13326,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 01/10/2026</t>
+          <t xml:space="preserve">Vigencia: 21/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (23/10/2026 05:47)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -11956,7 +11956,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 14/10/2026</t>
+          <t xml:space="preserve">Vigencia: 23/10/2026</t>
         </is>
       </c>
     </row>
@@ -12133,27 +12133,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HARINA MASA MADRE S/GLUTE X 400 G</t>
+          <t xml:space="preserve">HARINA 000 MASA MADRE 10x1</t>
         </is>
       </c>
       <c r="C11" s="4">
         <v>10</v>
       </c>
       <c r="D11" s="5">
-        <v>19326.25</v>
+        <v>13357.93</v>
       </c>
       <c r="E11" s="5">
         <f>IF(C11&gt;0,D11/C11,"")</f>
-        <v>1932.625</v>
+        <v>1335.7930000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4">
-        <v>3626034</v>
+        <v>3626033</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PREM PAN DE QUESO S/GLUTEN X 300 G</t>
+          <t xml:space="preserve">HARINA MASA MADRE S/GLUTE X 400 G</t>
         </is>
       </c>
       <c r="C12" s="4">
@@ -12169,21 +12169,41 @@
     </row>
     <row r="13">
       <c r="A13" s="4">
-        <v>3626040</v>
+        <v>3626034</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HARINA 00 PIZZA NAPOLETANA 10 X 1  KG</t>
+          <t xml:space="preserve">PREM PAN DE QUESO S/GLUTEN X 300 G</t>
         </is>
       </c>
       <c r="C13" s="4">
         <v>10</v>
       </c>
       <c r="D13" s="5">
-        <v>25610.4</v>
+        <v>19326.25</v>
       </c>
       <c r="E13" s="5">
         <f>IF(C13&gt;0,D13/C13,"")</f>
+        <v>1932.625</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>3626040</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HARINA 00 PIZZA NAPOLETANA 10 X 1  KG</t>
+        </is>
+      </c>
+      <c r="C14" s="4">
+        <v>10</v>
+      </c>
+      <c r="D14" s="5">
+        <v>25610.4</v>
+      </c>
+      <c r="E14" s="5">
+        <f>IF(C14&gt;0,D14/C14,"")</f>
         <v>2561.04</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (24/10/2026 05:44)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -8636,10 +8636,15 @@
           <t xml:space="preserve">YOG.FIRME DES. FRUT. POTE X 190G. ILOLAY</t>
         </is>
       </c>
-      <c r="C54" s="4"/>
-      <c r="D54" s="5"/>
+      <c r="C54" s="4">
+        <v>20</v>
+      </c>
+      <c r="D54" s="5">
+        <v>24788.79</v>
+      </c>
       <c r="E54" s="5">
-        <v>1239.44</v>
+        <f>IF(C54&gt;0,D54/C54,"")</f>
+        <v>1239.4395</v>
       </c>
     </row>
     <row r="55">

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (26/10/2026 05:55)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -9066,10 +9066,15 @@
           <t xml:space="preserve">TETRATOP PROTEINA VAINILLA X220GR ILOLAY</t>
         </is>
       </c>
-      <c r="C78" s="4"/>
-      <c r="D78" s="5"/>
+      <c r="C78" s="4">
+        <v>24</v>
+      </c>
+      <c r="D78" s="5">
+        <v>54777.28</v>
+      </c>
       <c r="E78" s="5">
-        <v>2282.39</v>
+        <f>IF(C78&gt;0,D78/C78,"")</f>
+        <v>2282.3866666666668</v>
       </c>
     </row>
     <row r="79">

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (28/10/2026 06:00)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -5951,9 +5951,14 @@
           <t xml:space="preserve">FLYNN PAFF BOLSA SURTIDA 8X8GR</t>
         </is>
       </c>
-      <c r="C168" s="4"/>
-      <c r="D168" s="5"/>
+      <c r="C168" s="4">
+        <v>8</v>
+      </c>
+      <c r="D168" s="5">
+        <v>61993.04</v>
+      </c>
       <c r="E168" s="5">
+        <f>IF(C168&gt;0,D168/C168,"")</f>
         <v>7749.13</v>
       </c>
     </row>
@@ -18241,7 +18246,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 27/10/2026</t>
+          <t xml:space="preserve">Vigencia: 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -19534,41 +19539,61 @@
     </row>
     <row r="67">
       <c r="A67" s="4">
-        <v>39014884</v>
+        <v>39014882</v>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DR LEMON RED BERRIES 5% 4x6x473</t>
+          <t xml:space="preserve">Gancia LIMA LIMON ONE 4x6x473</t>
         </is>
       </c>
       <c r="C67" s="4">
         <v>24</v>
       </c>
       <c r="D67" s="5">
-        <v>46766.89</v>
+        <v>42932.74</v>
       </c>
       <c r="E67" s="5">
         <f>IF(C67&gt;0,D67/C67,"")</f>
-        <v>1948.6204166666666</v>
+        <v>1788.8641666666665</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4">
-        <v>39014996</v>
+        <v>39014884</v>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Martini Rosso 16° 12x995ml</t>
+          <t xml:space="preserve">DR LEMON RED BERRIES 5% 4x6x473</t>
         </is>
       </c>
       <c r="C68" s="4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D68" s="5">
-        <v>93259.44</v>
+        <v>46766.89</v>
       </c>
       <c r="E68" s="5">
         <f>IF(C68&gt;0,D68/C68,"")</f>
+        <v>1948.6204166666666</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4">
+        <v>39014996</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Martini Rosso 16° 12x995ml</t>
+        </is>
+      </c>
+      <c r="C69" s="4">
+        <v>12</v>
+      </c>
+      <c r="D69" s="5">
+        <v>93259.44</v>
+      </c>
+      <c r="E69" s="5">
+        <f>IF(C69&gt;0,D69/C69,"")</f>
         <v>7771.62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (28/10/2026 09:34)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -2460,78 +2460,74 @@
     </row>
     <row r="95">
       <c r="A95" s="4">
-        <v>1506523</v>
+        <v>1506286</v>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Serv Elite Int Plus SH X250/72</t>
+          <t xml:space="preserve">Paños Maxwipe x70 Rollo x88/6</t>
         </is>
       </c>
       <c r="C95" s="4"/>
       <c r="D95" s="4">
-        <v>72</v>
+        <v>6</v>
       </c>
       <c r="E95" s="5">
-        <v>63234.6</v>
+        <v>18455.39</v>
       </c>
       <c r="F95" s="5">
         <f>IF(D95&gt;0,E95/D95,"")</f>
-        <v>878.25833333333333</v>
+        <v>3075.8983333333331</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4">
-        <v>1509232</v>
+        <v>1506385</v>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC NOBLE 40P x3/10</t>
-        </is>
-      </c>
-      <c r="C96" s="4">
-        <v>48</v>
-      </c>
+          <t xml:space="preserve">Paños Maxwipe 60 Q X50/12 Blanco</t>
+        </is>
+      </c>
+      <c r="C96" s="4"/>
       <c r="D96" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E96" s="5">
-        <v>15947.45</v>
+        <v>48228.18</v>
       </c>
       <c r="F96" s="5">
         <f>IF(D96&gt;0,E96/D96,"")</f>
-        <v>1594.7450000000001</v>
+        <v>4019.015</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4">
-        <v>1509243</v>
+        <v>1506523</v>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PH NOBLE HS 30M X4/12</t>
-        </is>
-      </c>
-      <c r="C97" s="4">
-        <v>60</v>
-      </c>
+          <t xml:space="preserve">Serv Elite Int Plus SH X250/72</t>
+        </is>
+      </c>
+      <c r="C97" s="4"/>
       <c r="D97" s="4">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="E97" s="5">
-        <v>21596.33</v>
+        <v>63234.6</v>
       </c>
       <c r="F97" s="5">
         <f>IF(D97&gt;0,E97/D97,"")</f>
-        <v>1799.6941666666669</v>
+        <v>878.25833333333333</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4">
-        <v>1509244</v>
+        <v>1509232</v>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PH NOBLE HS 30X6</t>
+          <t xml:space="preserve">RC NOBLE 40P x3/10</t>
         </is>
       </c>
       <c r="C98" s="4">
@@ -2541,342 +2537,342 @@
         <v>10</v>
       </c>
       <c r="E98" s="5">
-        <v>26082.47</v>
+        <v>15947.45</v>
       </c>
       <c r="F98" s="5">
         <f>IF(D98&gt;0,E98/D98,"")</f>
-        <v>2608.2470000000003</v>
+        <v>1594.7450000000001</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4">
-        <v>1509245</v>
+        <v>1509243</v>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PH NOBLE DH 30x4/10</t>
+          <t xml:space="preserve">PH NOBLE HS 30M X4/12</t>
         </is>
       </c>
       <c r="C99" s="4">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="D99" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E99" s="5">
-        <v>28089.53</v>
+        <v>21596.33</v>
       </c>
       <c r="F99" s="5">
         <f>IF(D99&gt;0,E99/D99,"")</f>
-        <v>2808.953</v>
+        <v>1799.6941666666669</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4">
-        <v>1509749</v>
+        <v>1509244</v>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PD ladysoft clasicos 20x30</t>
+          <t xml:space="preserve">PH NOBLE HS 30X6</t>
         </is>
       </c>
       <c r="C100" s="4">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="D100" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E100" s="5">
-        <v>47205.4</v>
+        <v>26082.47</v>
       </c>
       <c r="F100" s="5">
         <f>IF(D100&gt;0,E100/D100,"")</f>
-        <v>1573.5133333333333</v>
+        <v>2608.2470000000003</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4">
-        <v>1509750</v>
+        <v>1509245</v>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PD LADYSOFT CLASICOS 56x10</t>
+          <t xml:space="preserve">PH NOBLE DH 30x4/10</t>
         </is>
       </c>
       <c r="C101" s="4">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="D101" s="4">
         <v>10</v>
       </c>
       <c r="E101" s="5">
-        <v>41386.85</v>
+        <v>28089.53</v>
       </c>
       <c r="F101" s="5">
         <f>IF(D101&gt;0,E101/D101,"")</f>
-        <v>4138.6849999999995</v>
+        <v>2808.953</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4">
-        <v>1509755</v>
+        <v>1509749</v>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF UD T/SECA LADYSOFT ULTRA PROTECT 8</t>
+          <t xml:space="preserve">PD ladysoft clasicos 20x30</t>
         </is>
       </c>
       <c r="C102" s="4">
         <v>60</v>
       </c>
       <c r="D102" s="4">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E102" s="5">
-        <v>58063.82</v>
+        <v>47205.4</v>
       </c>
       <c r="F102" s="5">
         <f>IF(D102&gt;0,E102/D102,"")</f>
-        <v>1451.5955</v>
+        <v>1573.5133333333333</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4">
-        <v>1509756</v>
+        <v>1509750</v>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF UD T/SECA LADYSOFT UL PRT 16u</t>
+          <t xml:space="preserve">PD LADYSOFT CLASICOS 56x10</t>
         </is>
       </c>
       <c r="C103" s="4">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="D103" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E103" s="5">
-        <v>56475.9</v>
+        <v>41386.85</v>
       </c>
       <c r="F103" s="5">
         <f>IF(D103&gt;0,E103/D103,"")</f>
-        <v>2823.795</v>
+        <v>4138.6849999999995</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4">
-        <v>1509757</v>
+        <v>1509755</v>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF UD T/SECA LADYSOFT UL PTEC 24u</t>
+          <t xml:space="preserve">TF UD T/SECA LADYSOFT ULTRA PROTECT 8</t>
         </is>
       </c>
       <c r="C104" s="4">
         <v>60</v>
       </c>
       <c r="D104" s="4">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="E104" s="5">
-        <v>60502.23</v>
+        <v>58063.82</v>
       </c>
       <c r="F104" s="5">
         <f>IF(D104&gt;0,E104/D104,"")</f>
-        <v>4033.4820000000004</v>
+        <v>1451.5955</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4">
-        <v>1509758</v>
+        <v>1509756</v>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF UD T/SUAVE EXT ALGO 8X40</t>
+          <t xml:space="preserve">TF UD T/SECA LADYSOFT UL PRT 16u</t>
         </is>
       </c>
       <c r="C105" s="4">
         <v>60</v>
       </c>
       <c r="D105" s="4">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E105" s="5">
-        <v>54001.88</v>
+        <v>56475.9</v>
       </c>
       <c r="F105" s="5">
         <f>IF(D105&gt;0,E105/D105,"")</f>
-        <v>1350.047</v>
+        <v>2823.795</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="4">
-        <v>1509759</v>
+        <v>1509757</v>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF UD T/SUAVE EXT ALG 16x20</t>
+          <t xml:space="preserve">TF UD T/SECA LADYSOFT UL PTEC 24u</t>
         </is>
       </c>
       <c r="C106" s="4">
         <v>60</v>
       </c>
       <c r="D106" s="4">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E106" s="5">
-        <v>51563.15</v>
+        <v>60502.23</v>
       </c>
       <c r="F106" s="5">
         <f>IF(D106&gt;0,E106/D106,"")</f>
-        <v>2578.1575000000003</v>
+        <v>4033.4820000000004</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="4">
-        <v>1509760</v>
+        <v>1509758</v>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TD UF T/Suave Ladysoft EXT ALGODÓN 24x15</t>
+          <t xml:space="preserve">TF UD T/SUAVE EXT ALGO 8X40</t>
         </is>
       </c>
       <c r="C107" s="4">
         <v>60</v>
       </c>
       <c r="D107" s="4">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="E107" s="5">
-        <v>55018.2</v>
+        <v>54001.88</v>
       </c>
       <c r="F107" s="5">
         <f>IF(D107&gt;0,E107/D107,"")</f>
-        <v>3667.8799999999997</v>
+        <v>1350.047</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4">
-        <v>1509761</v>
+        <v>1509759</v>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF LADYSOFT COMFORT EXT ALGODON 8x54</t>
+          <t xml:space="preserve">TF UD T/SUAVE EXT ALG 16x20</t>
         </is>
       </c>
       <c r="C108" s="4">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D108" s="4">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E108" s="5">
-        <v>51959.99</v>
+        <v>51563.15</v>
       </c>
       <c r="F108" s="5">
         <f>IF(D108&gt;0,E108/D108,"")</f>
-        <v>962.222037037037</v>
+        <v>2578.1575000000003</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4">
-        <v>1509762</v>
+        <v>1509760</v>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF NOCTUR EXT A 8x32</t>
+          <t xml:space="preserve">TD UF T/Suave Ladysoft EXT ALGODÓN 24x15</t>
         </is>
       </c>
       <c r="C109" s="4">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D109" s="4">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E109" s="5">
-        <v>45387.27</v>
+        <v>55018.2</v>
       </c>
       <c r="F109" s="5">
         <f>IF(D109&gt;0,E109/D109,"")</f>
-        <v>1418.3521875</v>
+        <v>3667.8799999999997</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4">
-        <v>1509763</v>
+        <v>1509761</v>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF Nocturna EXT ALGODON 16X16</t>
+          <t xml:space="preserve">TF LADYSOFT COMFORT EXT ALGODON 8x54</t>
         </is>
       </c>
       <c r="C110" s="4">
+        <v>50</v>
+      </c>
+      <c r="D110" s="4">
         <v>54</v>
       </c>
-      <c r="D110" s="4">
-        <v>16</v>
-      </c>
       <c r="E110" s="5">
-        <v>43851.46</v>
+        <v>51959.99</v>
       </c>
       <c r="F110" s="5">
         <f>IF(D110&gt;0,E110/D110,"")</f>
-        <v>2740.71625</v>
+        <v>962.222037037037</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4">
-        <v>1509764</v>
+        <v>1509762</v>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF NORMAL T/SUAVE EXT ALGODON 8x54</t>
+          <t xml:space="preserve">TF NOCTUR EXT A 8x32</t>
         </is>
       </c>
       <c r="C111" s="4">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D111" s="4">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E111" s="5">
-        <v>54222.36</v>
+        <v>45387.27</v>
       </c>
       <c r="F111" s="5">
         <f>IF(D111&gt;0,E111/D111,"")</f>
-        <v>1004.1177777777777</v>
+        <v>1418.3521875</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4">
-        <v>1509765</v>
+        <v>1509763</v>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF NORMALT/SUAVE EXT ALG 16x27</t>
+          <t xml:space="preserve">TF Nocturna EXT ALGODON 16X16</t>
         </is>
       </c>
       <c r="C112" s="4">
         <v>54</v>
       </c>
       <c r="D112" s="4">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E112" s="5">
-        <v>54303.52</v>
+        <v>43851.46</v>
       </c>
       <c r="F112" s="5">
         <f>IF(D112&gt;0,E112/D112,"")</f>
-        <v>2011.2414814814813</v>
+        <v>2740.71625</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4">
-        <v>1509766</v>
+        <v>1509764</v>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF T/SECA NORMAL MAS PROTECC 8x54</t>
+          <t xml:space="preserve">TF NORMAL T/SUAVE EXT ALGODON 8x54</t>
         </is>
       </c>
       <c r="C113" s="4">
@@ -2886,43 +2882,43 @@
         <v>54</v>
       </c>
       <c r="E113" s="5">
-        <v>59838.63</v>
+        <v>54222.36</v>
       </c>
       <c r="F113" s="5">
         <f>IF(D113&gt;0,E113/D113,"")</f>
-        <v>1108.1227777777776</v>
+        <v>1004.1177777777777</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4">
-        <v>1509767</v>
+        <v>1509765</v>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF UD TSUAVE ACTIVE 8X40</t>
+          <t xml:space="preserve">TF NORMALT/SUAVE EXT ALG 16x27</t>
         </is>
       </c>
       <c r="C114" s="4">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D114" s="4">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="E114" s="5">
-        <v>65673.74</v>
+        <v>54303.52</v>
       </c>
       <c r="F114" s="5">
         <f>IF(D114&gt;0,E114/D114,"")</f>
-        <v>1641.8435000000002</v>
+        <v>2011.2414814814813</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4">
-        <v>1509768</v>
+        <v>1509766</v>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TF NORMAL T/SUAVE PIEL SENSIBLE 8x54</t>
+          <t xml:space="preserve">TF T/SECA NORMAL MAS PROTECC 8x54</t>
         </is>
       </c>
       <c r="C115" s="4">
@@ -2932,66 +2928,112 @@
         <v>54</v>
       </c>
       <c r="E115" s="5">
-        <v>63726.79</v>
+        <v>59838.63</v>
       </c>
       <c r="F115" s="5">
         <f>IF(D115&gt;0,E115/D115,"")</f>
-        <v>1180.1257407407409</v>
+        <v>1108.1227777777776</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4">
-        <v>1509769</v>
+        <v>1509767</v>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PD RESPIRABLES 100/12</t>
+          <t xml:space="preserve">TF UD TSUAVE ACTIVE 8X40</t>
         </is>
       </c>
       <c r="C116" s="4">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D116" s="4">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="E116" s="5">
-        <v>76814.97</v>
+        <v>65673.74</v>
       </c>
       <c r="F116" s="5">
         <f>IF(D116&gt;0,E116/D116,"")</f>
-        <v>6401.2475</v>
+        <v>1641.8435000000002</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4">
-        <v>1509916</v>
+        <v>1509768</v>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PD LADYSOFT UD RESPIRABLE S/ALAS X20/30</t>
-        </is>
-      </c>
-      <c r="C117" s="4"/>
+          <t xml:space="preserve">TF NORMAL T/SUAVE PIEL SENSIBLE 8x54</t>
+        </is>
+      </c>
+      <c r="C117" s="4">
+        <v>54</v>
+      </c>
       <c r="D117" s="4">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="E117" s="5">
-        <v>47622.19</v>
+        <v>63726.79</v>
       </c>
       <c r="F117" s="5">
         <f>IF(D117&gt;0,E117/D117,"")</f>
+        <v>1180.1257407407409</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4">
+        <v>1509769</v>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PD RESPIRABLES 100/12</t>
+        </is>
+      </c>
+      <c r="C118" s="4">
+        <v>50</v>
+      </c>
+      <c r="D118" s="4">
+        <v>12</v>
+      </c>
+      <c r="E118" s="5">
+        <v>76814.97</v>
+      </c>
+      <c r="F118" s="5">
+        <f>IF(D118&gt;0,E118/D118,"")</f>
+        <v>6401.2475</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4">
+        <v>1509916</v>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PD LADYSOFT UD RESPIRABLE S/ALAS X20/30</t>
+        </is>
+      </c>
+      <c r="C119" s="4"/>
+      <c r="D119" s="4">
+        <v>30</v>
+      </c>
+      <c r="E119" s="5">
+        <v>47622.19</v>
+      </c>
+      <c r="F119" s="5">
+        <f>IF(D119&gt;0,E119/D119,"")</f>
         <v>1587.4063333333334</v>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="6" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">* 1503121 TH Babysec Premium 50/10: En el sistema el precio Pack figura 10 veces mas alto. Se toma el precio Unidad del sistema como precio del bulto.</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="6" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">* 1504739 PL BABYSEC ULTRA M 26/8: El sistema lo carga con 6 por bulto; segun la tabla de logistica y la descripcion (26/8) son 8. Se toman 8.</t>
         </is>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (29/10/2026 06:02)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -351,7 +351,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 20/10/2026</t>
+          <t xml:space="preserve">Vigencia: 29/10/2026</t>
         </is>
       </c>
     </row>
@@ -18288,7 +18288,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 28/10/2026</t>
+          <t xml:space="preserve">Vigencia: 29/10/2026</t>
         </is>
       </c>
     </row>
@@ -19581,61 +19581,81 @@
     </row>
     <row r="67">
       <c r="A67" s="4">
-        <v>39014882</v>
+        <v>39014866</v>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gancia LIMA LIMON ONE 4x6x473</t>
+          <t xml:space="preserve">1882 FERNET CON POMELO 7 473mlx6x4</t>
         </is>
       </c>
       <c r="C67" s="4">
         <v>24</v>
       </c>
       <c r="D67" s="5">
-        <v>42932.74</v>
+        <v>40363.42</v>
       </c>
       <c r="E67" s="5">
         <f>IF(C67&gt;0,D67/C67,"")</f>
-        <v>1788.8641666666665</v>
+        <v>1681.8091666666667</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4">
-        <v>39014884</v>
+        <v>39014882</v>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DR LEMON RED BERRIES 5% 4x6x473</t>
+          <t xml:space="preserve">Gancia LIMA LIMON ONE 4x6x473</t>
         </is>
       </c>
       <c r="C68" s="4">
         <v>24</v>
       </c>
       <c r="D68" s="5">
-        <v>46766.89</v>
+        <v>42932.74</v>
       </c>
       <c r="E68" s="5">
         <f>IF(C68&gt;0,D68/C68,"")</f>
-        <v>1948.6204166666666</v>
+        <v>1788.8641666666665</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4">
-        <v>39014996</v>
+        <v>39014884</v>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Martini Rosso 16° 12x995ml</t>
+          <t xml:space="preserve">DR LEMON RED BERRIES 5% 4x6x473</t>
         </is>
       </c>
       <c r="C69" s="4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D69" s="5">
-        <v>93259.44</v>
+        <v>46766.89</v>
       </c>
       <c r="E69" s="5">
         <f>IF(C69&gt;0,D69/C69,"")</f>
+        <v>1948.6204166666666</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4">
+        <v>39014996</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Martini Rosso 16° 12x995ml</t>
+        </is>
+      </c>
+      <c r="C70" s="4">
+        <v>12</v>
+      </c>
+      <c r="D70" s="5">
+        <v>93259.44</v>
+      </c>
+      <c r="E70" s="5">
+        <f>IF(C70&gt;0,D70/C70,"")</f>
         <v>7771.62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (30/10/2026 06:02)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -7584,14 +7584,14 @@
         </is>
       </c>
       <c r="C258" s="4">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D258" s="5">
-        <v>229281.25</v>
+        <v>128970.71</v>
       </c>
       <c r="E258" s="5">
         <f>IF(C258&gt;0,D258/C258,"")</f>
-        <v>7165.0390625</v>
+        <v>7165.0394444444446</v>
       </c>
     </row>
     <row r="259">

</xml_diff>

<commit_message>
Listas de precios actualizadas desde Gescom (31/10/2026 05:53)
</commit_message>
<xml_diff>
--- a/Listas de precios LP - ELEBES.xlsx
+++ b/Listas de precios LP - ELEBES.xlsx
@@ -16448,7 +16448,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia: 06/10/2026</t>
+          <t xml:space="preserve">Vigencia: 31/10/2026</t>
         </is>
       </c>
     </row>
@@ -16671,31 +16671,26 @@
     </row>
     <row r="15">
       <c r="A15" s="4">
-        <v>4180154</v>
+        <v>4180153</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maní c Sal s/piel 100g x 15 u</t>
-        </is>
-      </c>
-      <c r="C15" s="4">
-        <v>15</v>
-      </c>
-      <c r="D15" s="5">
-        <v>12574.27</v>
-      </c>
+          <t xml:space="preserve">Mani Chef Sabor Asado 15x80g</t>
+        </is>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="5"/>
       <c r="E15" s="5">
-        <f>IF(C15&gt;0,D15/C15,"")</f>
-        <v>838.28466666666668</v>
+        <v>13394.91</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4">
-        <v>4180155</v>
+        <v>4180154</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maní Sal con Piel 100G X 15u</t>
+          <t xml:space="preserve">Maní c Sal s/piel 100g x 15 u</t>
         </is>
       </c>
       <c r="C16" s="4">
@@ -16711,251 +16706,286 @@
     </row>
     <row r="17">
       <c r="A17" s="4">
-        <v>4180203</v>
+        <v>4180155</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maní Tostado con Cáscara 175G</t>
-        </is>
-      </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="5"/>
+          <t xml:space="preserve">Maní Sal con Piel 100G X 15u</t>
+        </is>
+      </c>
+      <c r="C17" s="4">
+        <v>15</v>
+      </c>
+      <c r="D17" s="5">
+        <v>12574.27</v>
+      </c>
       <c r="E17" s="5">
-        <v>18804.44</v>
+        <f>IF(C17&gt;0,D17/C17,"")</f>
+        <v>838.28466666666668</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4">
-        <v>41800103</v>
+        <v>4180169</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mani c chocolate 15 x 80 grs</t>
-        </is>
-      </c>
-      <c r="C18" s="4">
-        <v>15</v>
-      </c>
-      <c r="D18" s="5">
-        <v>21618.74</v>
-      </c>
+          <t xml:space="preserve">Mani Sal Marina 200g  x12u</t>
+        </is>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="5"/>
       <c r="E18" s="5">
-        <f>IF(C18&gt;0,D18/C18,"")</f>
-        <v>1441.2493333333334</v>
+        <v>23866.42</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4">
-        <v>41800104</v>
+        <v>4180203</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GarrapiÑada 20 x 80 grs x 20 u</t>
-        </is>
-      </c>
-      <c r="C19" s="4">
-        <v>20</v>
-      </c>
-      <c r="D19" s="5">
-        <v>13117.49</v>
-      </c>
+          <t xml:space="preserve">Maní Tostado con Cáscara 175G</t>
+        </is>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="5"/>
       <c r="E19" s="5">
-        <f>IF(C19&gt;0,D19/C19,"")</f>
-        <v>655.8745</v>
+        <v>18804.44</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4">
-        <v>41800131</v>
+        <v>41800103</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pasta de Mani cruchy  350x12gr</t>
+          <t xml:space="preserve">Mani c chocolate 15 x 80 grs</t>
         </is>
       </c>
       <c r="C20" s="4">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D20" s="5">
-        <v>85078.8</v>
+        <v>21618.74</v>
       </c>
       <c r="E20" s="5">
         <f>IF(C20&gt;0,D20/C20,"")</f>
-        <v>7089.9000000000005</v>
+        <v>1441.2493333333334</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4">
-        <v>41800152</v>
+        <v>41800104</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mani Frito Mk  SIN PIEL 20 x350 gr</t>
-        </is>
-      </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="5"/>
+          <t xml:space="preserve">GarrapiÑada 20 x 80 grs x 20 u</t>
+        </is>
+      </c>
+      <c r="C21" s="4">
+        <v>20</v>
+      </c>
+      <c r="D21" s="5">
+        <v>13117.49</v>
+      </c>
       <c r="E21" s="5">
-        <v>14454.47</v>
+        <f>IF(C21&gt;0,D21/C21,"")</f>
+        <v>655.8745</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4">
-        <v>41800208</v>
+        <v>41800131</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mani con cascara 10x400 gr</t>
+          <t xml:space="preserve">Pasta de Mani cruchy  350x12gr</t>
         </is>
       </c>
       <c r="C22" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D22" s="5">
-        <v>22706.91</v>
+        <v>85078.8</v>
       </c>
       <c r="E22" s="5">
         <f>IF(C22&gt;0,D22/C22,"")</f>
-        <v>2270.691</v>
+        <v>7089.9000000000005</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4">
-        <v>41800216</v>
+        <v>41800152</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mani c baño choco 15 x 80 grs</t>
-        </is>
-      </c>
-      <c r="C23" s="4">
-        <v>15</v>
-      </c>
-      <c r="D23" s="5">
-        <v>22110.08</v>
-      </c>
+          <t xml:space="preserve">Mani Frito Mk  SIN PIEL 20 x350 gr</t>
+        </is>
+      </c>
+      <c r="C23" s="4"/>
+      <c r="D23" s="5"/>
       <c r="E23" s="5">
-        <f>IF(C23&gt;0,D23/C23,"")</f>
-        <v>1474.0053333333335</v>
+        <v>14454.47</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4">
-        <v>41810134</v>
+        <v>41800208</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANI FRITO MK 1KG X 9</t>
-        </is>
-      </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="5"/>
+          <t xml:space="preserve">Mani con cascara 10x400 gr</t>
+        </is>
+      </c>
+      <c r="C24" s="4">
+        <v>10</v>
+      </c>
+      <c r="D24" s="5">
+        <v>22706.91</v>
+      </c>
       <c r="E24" s="5">
-        <v>54895.8</v>
+        <f>IF(C24&gt;0,D24/C24,"")</f>
+        <v>2270.691</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4">
-        <v>41810153</v>
+        <v>41800216</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANI FRITO C/ PIEL MK 20X350 GR</t>
-        </is>
-      </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="5"/>
+          <t xml:space="preserve">Mani c baño choco 15 x 80 grs</t>
+        </is>
+      </c>
+      <c r="C25" s="4">
+        <v>15</v>
+      </c>
+      <c r="D25" s="5">
+        <v>22110.08</v>
+      </c>
       <c r="E25" s="5">
-        <v>55511.5</v>
+        <f>IF(C25&gt;0,D25/C25,"")</f>
+        <v>1474.0053333333335</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4">
-        <v>41820115</v>
+        <v>41810134</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANI TOSTADO MK SIN SAL 20X350 GRS</t>
-        </is>
-      </c>
-      <c r="C26" s="4">
-        <v>20</v>
-      </c>
-      <c r="D26" s="5">
-        <v>55511.48</v>
-      </c>
+          <t xml:space="preserve">MANI FRITO MK 1KG X 9</t>
+        </is>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="5"/>
       <c r="E26" s="5">
-        <f>IF(C26&gt;0,D26/C26,"")</f>
-        <v>2775.574</v>
+        <v>54895.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4">
-        <v>41820116</v>
+        <v>41810153</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maní Tostado s/ Piel s/ Sal  100GR</t>
+          <t xml:space="preserve">MANI FRITO C/ PIEL MK 20X350 GR</t>
         </is>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5">
-        <v>12574.27</v>
+        <v>55511.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4">
-        <v>41820122</v>
+        <v>41820115</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANI TOSTADO 1KG X 9</t>
-        </is>
-      </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="5"/>
+          <t xml:space="preserve">MANI TOSTADO MK SIN SAL 20X350 GRS</t>
+        </is>
+      </c>
+      <c r="C28" s="4">
+        <v>20</v>
+      </c>
+      <c r="D28" s="5">
+        <v>55511.48</v>
+      </c>
       <c r="E28" s="5">
-        <v>54895.8</v>
+        <f>IF(C28&gt;0,D28/C28,"")</f>
+        <v>2775.574</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4">
-        <v>41860118</v>
+        <v>41820116</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASTA DE MANI MK NAT 6X1 KG</t>
-        </is>
-      </c>
-      <c r="C29" s="4">
-        <v>6</v>
-      </c>
-      <c r="D29" s="5">
-        <v>30562.08</v>
-      </c>
+          <t xml:space="preserve">Maní Tostado s/ Piel s/ Sal  100GR</t>
+        </is>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="5"/>
       <c r="E29" s="5">
-        <f>IF(C29&gt;0,D29/C29,"")</f>
-        <v>5093.68</v>
+        <v>12574.27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4">
+        <v>41820122</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MANI TOSTADO 1KG X 9</t>
+        </is>
+      </c>
+      <c r="C30" s="4"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5">
+        <v>54895.8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4">
+        <v>41860118</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASTA DE MANI MK NAT 6X1 KG</t>
+        </is>
+      </c>
+      <c r="C31" s="4">
+        <v>6</v>
+      </c>
+      <c r="D31" s="5">
+        <v>30562.08</v>
+      </c>
+      <c r="E31" s="5">
+        <f>IF(C31&gt;0,D31/C31,"")</f>
+        <v>5093.68</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4">
         <v>44834210</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">REDONDITOS CHOCOLATE  210 G 16U</t>
         </is>
       </c>
-      <c r="C30" s="4">
+      <c r="C32" s="4">
         <v>16</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D32" s="5">
         <v>26992.68</v>
       </c>
-      <c r="E30" s="5">
-        <f>IF(C30&gt;0,D30/C30,"")</f>
+      <c r="E32" s="5">
+        <f>IF(C32&gt;0,D32/C32,"")</f>
         <v>1687.0425</v>
       </c>
     </row>

</xml_diff>